<commit_message>
docs: regenerate document set and add zero-cost distribution runbook
</commit_message>
<xml_diff>
--- a/docs/PD_Code_Register_v1.0.xlsx
+++ b/docs/PD_Code_Register_v1.0.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="197">
   <si>
     <t>PulseDesk — Code Register</t>
   </si>
@@ -397,6 +397,9 @@
     <t>Preview server launch configuration</t>
   </si>
   <si>
+    <t>localhost:5173, localhost:5174</t>
+  </si>
+  <si>
     <t>README.md</t>
   </si>
   <si>
@@ -404,6 +407,180 @@
   </si>
   <si>
     <t>SDD §1</t>
+  </si>
+  <si>
+    <t>worker/src/index.js</t>
+  </si>
+  <si>
+    <t>Worker</t>
+  </si>
+  <si>
+    <t>CORS market-data relay plus the anonymous usage counter and private stats endpoint</t>
+  </si>
+  <si>
+    <t>/api/indices, /api/news, /api/hyped, /api/crypto, /api/sessions, /api/weather, /api/quotes, /api/fx, /api/lookup, /api/ping, /api/stats, /api/health</t>
+  </si>
+  <si>
+    <t>D1: events</t>
+  </si>
+  <si>
+    <t>FUN-034, FUN-036, FUN-037, SEC-011..SEC-014, NFR-011</t>
+  </si>
+  <si>
+    <t>SDD §10.1, §11</t>
+  </si>
+  <si>
+    <t>worker/wrangler.toml</t>
+  </si>
+  <si>
+    <t>Cloudflare Worker and D1 binding configuration</t>
+  </si>
+  <si>
+    <t>D1: pulsedesk</t>
+  </si>
+  <si>
+    <t>NFR-013</t>
+  </si>
+  <si>
+    <t>SDD §10.1</t>
+  </si>
+  <si>
+    <t>worker/schema.sql</t>
+  </si>
+  <si>
+    <t>Events table and indexes for the usage counter</t>
+  </si>
+  <si>
+    <t>FUN-036, SEC-012</t>
+  </si>
+  <si>
+    <t>SDD §11.1</t>
+  </si>
+  <si>
+    <t>web/src/web-bridge.js</t>
+  </si>
+  <si>
+    <t>Web</t>
+  </si>
+  <si>
+    <t>Browser implementation of window.pulse — fetch instead of IPC, localStorage instead of files</t>
+  </si>
+  <si>
+    <t>localStorage: pulse.*</t>
+  </si>
+  <si>
+    <t>FUN-034, FUN-035, FUN-036</t>
+  </si>
+  <si>
+    <t>SDD §10.2</t>
+  </si>
+  <si>
+    <t>web/src/install.js</t>
+  </si>
+  <si>
+    <t>Install prompt for Android/desktop and the Add to Home Screen hint for iOS</t>
+  </si>
+  <si>
+    <t>FUN-032</t>
+  </si>
+  <si>
+    <t>SDD §10.3</t>
+  </si>
+  <si>
+    <t>web/src/sw.js</t>
+  </si>
+  <si>
+    <t>Service worker — shell precache, network-only for market data</t>
+  </si>
+  <si>
+    <t>CacheStorage</t>
+  </si>
+  <si>
+    <t>FUN-033</t>
+  </si>
+  <si>
+    <t>web/src/web.css</t>
+  </si>
+  <si>
+    <t>Web and phone overrides on top of the shared stylesheet</t>
+  </si>
+  <si>
+    <t>NFR-012</t>
+  </si>
+  <si>
+    <t>web/src/manifest.webmanifest</t>
+  </si>
+  <si>
+    <t>Installability metadata, icons, theme and author credit</t>
+  </si>
+  <si>
+    <t>FUN-032, FUN-039</t>
+  </si>
+  <si>
+    <t>web/src/stats.html</t>
+  </si>
+  <si>
+    <t>Private usage dashboard — online now, opens per day, people, 30-day trend, country and platform split</t>
+  </si>
+  <si>
+    <t>/stats.html</t>
+  </si>
+  <si>
+    <t>reads /api/stats</t>
+  </si>
+  <si>
+    <t>FUN-037, SEC-011</t>
+  </si>
+  <si>
+    <t>SDD §11.2</t>
+  </si>
+  <si>
+    <t>tools/build-web.js</t>
+  </si>
+  <si>
+    <t>Assembles web/dist from the shared renderer, rewrites CSP, injects the bridge, emits icons and config</t>
+  </si>
+  <si>
+    <t>FUN-032, SEC-015</t>
+  </si>
+  <si>
+    <t>tools/gen-icons.js</t>
+  </si>
+  <si>
+    <t>Writes packaging icons from the runtime PNG encoder</t>
+  </si>
+  <si>
+    <t>FUN-038</t>
+  </si>
+  <si>
+    <t>SDD §10.4</t>
+  </si>
+  <si>
+    <t>.github/workflows/pages.yml</t>
+  </si>
+  <si>
+    <t>CI</t>
+  </si>
+  <si>
+    <t>Builds and deploys the web app to GitHub Pages on push</t>
+  </si>
+  <si>
+    <t>FUN-032, NFR-013</t>
+  </si>
+  <si>
+    <t>.github/workflows/release.yml</t>
+  </si>
+  <si>
+    <t>Builds the Windows installer and portable exe on a version tag and attaches them to the release</t>
+  </si>
+  <si>
+    <t>DEPLOY.md</t>
+  </si>
+  <si>
+    <t>Zero-cost distribution runbook for Pages, Releases, Cloudflare and the usage dashboard</t>
+  </si>
+  <si>
+    <t>SDD §10.5</t>
   </si>
   <si>
     <t>Metric</t>
@@ -1099,7 +1276,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1617,7 +1794,7 @@
         <v>126</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>52</v>
+        <v>127</v>
       </c>
       <c r="E20" s="8" t="s">
         <v>52</v>
@@ -1634,13 +1811,13 @@
     </row>
     <row r="21" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>52</v>
@@ -1652,9 +1829,373 @@
         <v>52</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H21" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="H26" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="H28" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="H30" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="H32" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="H34" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="H35" s="3" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1676,15 +2217,15 @@
   <sheetData>
     <row r="1" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>130</v>
+        <v>189</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>131</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>132</v>
+        <v>191</v>
       </c>
       <c r="B2" s="5">
         <f>COUNTA('Code Register'!A2:A400)</f>
@@ -1692,7 +2233,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>133</v>
+        <v>192</v>
       </c>
       <c r="B3" s="5">
         <f>COUNTIF('Code Register'!B2:B400,"Service")</f>
@@ -1700,7 +2241,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>134</v>
+        <v>193</v>
       </c>
       <c r="B4" s="5">
         <f>COUNTIF('Code Register'!B2:B400,"Renderer")</f>
@@ -1708,7 +2249,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>135</v>
+        <v>194</v>
       </c>
       <c r="B5" s="5">
         <f>COUNTIF('Code Register'!B2:B400,"Tooling")</f>
@@ -1716,7 +2257,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>136</v>
+        <v>195</v>
       </c>
       <c r="B6" s="5">
         <f>COUNTIF('Code Register'!H2:H400,"Done")</f>
@@ -1724,7 +2265,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>137</v>
+        <v>196</v>
       </c>
       <c r="B7" s="5">
         <f>ROUND(COUNTIF('Code Register'!H2:H400,"Done")/COUNTA('Code Register'!A2:A400)*100,1)</f>

</xml_diff>

<commit_message>
docs: regenerate document set at 54 functional requirements
</commit_message>
<xml_diff>
--- a/docs/PD_Code_Register_v1.0.xlsx
+++ b/docs/PD_Code_Register_v1.0.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="213">
   <si>
     <t>PulseDesk — Code Register</t>
   </si>
@@ -581,6 +581,54 @@
   </si>
   <si>
     <t>SDD §10.5</t>
+  </si>
+  <si>
+    <t>HOW-TO-PUBLISH.md</t>
+  </si>
+  <si>
+    <t>Click-by-click publishing guide with no command line, for a non-technical operator</t>
+  </si>
+  <si>
+    <t>FUN-053</t>
+  </si>
+  <si>
+    <t>SDD §10.6</t>
+  </si>
+  <si>
+    <t>INSTALL.md</t>
+  </si>
+  <si>
+    <t>End-user installation guide for phone, PC and browser, plus the holdings walkthrough</t>
+  </si>
+  <si>
+    <t>tools/bundle-worker.js</t>
+  </si>
+  <si>
+    <t>esbuild bundle of the worker into a single pasteable file</t>
+  </si>
+  <si>
+    <t>FUN-052</t>
+  </si>
+  <si>
+    <t>worker/dist/worker.js</t>
+  </si>
+  <si>
+    <t>Generated single-file worker for dashboard paste-deployment</t>
+  </si>
+  <si>
+    <t>run-pulsedesk.bat</t>
+  </si>
+  <si>
+    <t>Double-click launcher that installs dependencies on first run and starts the app</t>
+  </si>
+  <si>
+    <t>make-worker-file.bat</t>
+  </si>
+  <si>
+    <t>Double-click builder for the pasteable worker file</t>
+  </si>
+  <si>
+    <t>FUN-052, FUN-053</t>
   </si>
   <si>
     <t>Metric</t>
@@ -1276,7 +1324,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2196,6 +2244,162 @@
         <v>188</v>
       </c>
       <c r="H35" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="H36" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="G38" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="H38" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="G40" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="H40" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="H41" s="3" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2217,15 +2421,15 @@
   <sheetData>
     <row r="1" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>189</v>
+        <v>205</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>191</v>
+        <v>207</v>
       </c>
       <c r="B2" s="5">
         <f>COUNTA('Code Register'!A2:A400)</f>
@@ -2233,7 +2437,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>192</v>
+        <v>208</v>
       </c>
       <c r="B3" s="5">
         <f>COUNTIF('Code Register'!B2:B400,"Service")</f>
@@ -2241,7 +2445,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>193</v>
+        <v>209</v>
       </c>
       <c r="B4" s="5">
         <f>COUNTIF('Code Register'!B2:B400,"Renderer")</f>
@@ -2249,7 +2453,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="B5" s="5">
         <f>COUNTIF('Code Register'!B2:B400,"Tooling")</f>
@@ -2257,7 +2461,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>195</v>
+        <v>211</v>
       </c>
       <c r="B6" s="5">
         <f>COUNTIF('Code Register'!H2:H400,"Done")</f>
@@ -2265,7 +2469,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>196</v>
+        <v>212</v>
       </c>
       <c r="B7" s="5">
         <f>ROUND(COUNTIF('Code Register'!H2:H400,"Done")/COUNTA('Code Register'!A2:A400)*100,1)</f>

</xml_diff>

<commit_message>
docs: regenerate document set at 63 functional requirements
RTM now 63 functional / 16 security / 14 NFR; Code Register 41 rows;
Charter and SDD carry the mutual funds, stock chart, sector filter,
financial-hub weather and disclaimer scope added this round.
</commit_message>
<xml_diff>
--- a/docs/PD_Code_Register_v1.0.xlsx
+++ b/docs/PD_Code_Register_v1.0.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="217">
   <si>
     <t>PulseDesk — Code Register</t>
   </si>
@@ -184,16 +184,16 @@
     <t>main.js</t>
   </si>
   <si>
-    <t>Window lifecycle, tray, global shortcuts, IPC surface, tiered refresh orchestration</t>
-  </si>
-  <si>
-    <t>IPC: data:*, portfolio:*, settings:*, win:*</t>
+    <t>Window lifecycle, tray, global shortcuts, IPC surface (incl. search:history), tiered refresh orchestration including funds and financial-hub cities</t>
+  </si>
+  <si>
+    <t>IPC: data:*, portfolio:*, settings:*, win:*, search:*</t>
   </si>
   <si>
     <t>settings.json</t>
   </si>
   <si>
-    <t>FUN-025..FUN-029, SEC-004, SEC-005</t>
+    <t>FUN-025..FUN-029, FUN-055, FUN-058, FUN-062, SEC-004, SEC-005</t>
   </si>
   <si>
     <t>SDD §3</t>
@@ -202,7 +202,7 @@
     <t>preload.js</t>
   </si>
   <si>
-    <t>contextBridge API exposed to the renderer as window.pulse</t>
+    <t>contextBridge API exposed to the renderer as window.pulse, including history()</t>
   </si>
   <si>
     <t>IPC allowlist</t>
@@ -229,13 +229,13 @@
     <t>src/services/stocks.js</t>
   </si>
   <si>
-    <t>Yahoo chart normalisation, Stooq fallback, index basket, FX cross, hype scoring</t>
-  </si>
-  <si>
-    <t>FUN-001..FUN-003, FUN-008, FUN-020, NFR-010</t>
-  </si>
-  <si>
-    <t>SDD §4.1, §4.2</t>
+    <t>Yahoo chart normalisation, Stooq fallback, index basket, FX cross, hype scoring, sector-tagged popular list, 1D-5Y history series</t>
+  </si>
+  <si>
+    <t>FUN-001..FUN-003, FUN-008, FUN-020, FUN-058, FUN-060, NFR-010</t>
+  </si>
+  <si>
+    <t>SDD §4.1, §4.2, §4.11, §4.13</t>
   </si>
   <si>
     <t>src/services/sentiment.js</t>
@@ -277,10 +277,10 @@
     <t>src/services/weather.js</t>
   </si>
   <si>
-    <t>IP geolocation chain, Open-Meteo forecast, air quality, weather-code mapping</t>
-  </si>
-  <si>
-    <t>FUN-023, FUN-024</t>
+    <t>IP geolocation chain, Open-Meteo forecast, air quality, weather-code mapping, six-city financial-hub snapshot</t>
+  </si>
+  <si>
+    <t>FUN-023, FUN-024, FUN-062</t>
   </si>
   <si>
     <t>SDD §4.8</t>
@@ -304,15 +304,27 @@
     <t>src/services/market.js</t>
   </si>
   <si>
-    <t>Exchange session clocks, breadth calculation, composite pulse score</t>
-  </si>
-  <si>
-    <t>FUN-021, FUN-022</t>
+    <t>Exchange session clocks with open-now/closes-in wording, breadth calculation, composite pulse score</t>
+  </si>
+  <si>
+    <t>FUN-021, FUN-022, FUN-063</t>
   </si>
   <si>
     <t>SDD §4.7</t>
   </si>
   <si>
+    <t>src/services/mutualfunds.js</t>
+  </si>
+  <si>
+    <t>Curated Direct-Growth mutual fund NAVs from mfapi.in by pinned scheme code, with day/month/year change</t>
+  </si>
+  <si>
+    <t>FUN-055, FUN-056, SEC-016</t>
+  </si>
+  <si>
+    <t>SDD §4.12</t>
+  </si>
+  <si>
     <t>src/services/icon.js</t>
   </si>
   <si>
@@ -328,10 +340,10 @@
     <t>src/renderer/index.html</t>
   </si>
   <si>
-    <t>Dashboard markup, CSP declaration, modal shells</t>
-  </si>
-  <si>
-    <t>SEC-002, NFR-006</t>
+    <t>Dashboard markup, CSP declaration, modal shells including the stock chart and all-scanned-stocks modals</t>
+  </si>
+  <si>
+    <t>SEC-002, NFR-006, FUN-057, FUN-058</t>
   </si>
   <si>
     <t>SDD §5.1</t>
@@ -340,10 +352,10 @@
     <t>src/renderer/styles.css</t>
   </si>
   <si>
-    <t>Glass finance theme, fixed-height card grid, responsive and compact layouts</t>
-  </si>
-  <si>
-    <t>FUN-031, NFR-006, NFR-007</t>
+    <t>Glass finance theme, fixed-height card grid, chart/modal styling, responsive, compact and mobile-touch layouts</t>
+  </si>
+  <si>
+    <t>FUN-031, NFR-006, NFR-007, NFR-012</t>
   </si>
   <si>
     <t>SDD §5.2</t>
@@ -352,10 +364,10 @@
     <t>src/renderer/app.js</t>
   </si>
   <si>
-    <t>Formatting helpers, SVG sparkline/donut builders, section renderers, event wiring</t>
-  </si>
-  <si>
-    <t>FUN-009, FUN-015, FUN-030, SEC-003</t>
+    <t>Formatting helpers, SVG sparkline/donut/chart builders, likely-call heuristic, related-news matcher, section renderers, event wiring</t>
+  </si>
+  <si>
+    <t>FUN-009, FUN-015, FUN-030, FUN-054, FUN-057..FUN-061, SEC-003</t>
   </si>
   <si>
     <t>SDD §5.3</t>
@@ -418,13 +430,13 @@
     <t>CORS market-data relay plus the anonymous usage counter and private stats endpoint</t>
   </si>
   <si>
-    <t>/api/indices, /api/news, /api/hyped, /api/crypto, /api/sessions, /api/weather, /api/quotes, /api/fx, /api/lookup, /api/ping, /api/stats, /api/health</t>
+    <t>/api/indices, /api/news, /api/hyped, /api/popular, /api/funds, /api/crypto, /api/sessions, /api/weather, /api/cities, /api/quotes, /api/fx, /api/lookup, /api/search, /api/price-at, /api/history, /api/ping, /api/stats, /api/health</t>
   </si>
   <si>
     <t>D1: events</t>
   </si>
   <si>
-    <t>FUN-034, FUN-036, FUN-037, SEC-011..SEC-014, NFR-011</t>
+    <t>FUN-034, FUN-036, FUN-037, FUN-055, FUN-058, FUN-062, SEC-011..SEC-014, SEC-016, NFR-011</t>
   </si>
   <si>
     <t>SDD §10.1, §11</t>
@@ -463,13 +475,13 @@
     <t>Web</t>
   </si>
   <si>
-    <t>Browser implementation of window.pulse — fetch instead of IPC, localStorage instead of files</t>
+    <t>Browser implementation of window.pulse — fetch instead of IPC, localStorage instead of files, including funds/cities/history</t>
   </si>
   <si>
     <t>localStorage: pulse.*</t>
   </si>
   <si>
-    <t>FUN-034, FUN-035, FUN-036</t>
+    <t>FUN-034, FUN-035, FUN-036, FUN-055, FUN-058, FUN-062</t>
   </si>
   <si>
     <t>SDD §10.2</t>
@@ -1324,7 +1336,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1680,7 +1692,7 @@
         <v>103</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>104</v>
@@ -1758,22 +1770,22 @@
         <v>115</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>116</v>
       </c>
       <c r="D17" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="E17" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F17" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>119</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>33</v>
@@ -1781,25 +1793,25 @@
     </row>
     <row r="18" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B18" s="8" t="s">
         <v>27</v>
       </c>
       <c r="C18" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="D18" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="D18" s="8" t="s">
-        <v>52</v>
-      </c>
       <c r="E18" s="8" t="s">
         <v>52</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>52</v>
+        <v>122</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>33</v>
@@ -1807,13 +1819,13 @@
     </row>
     <row r="19" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>27</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>52</v>
@@ -1825,7 +1837,7 @@
         <v>52</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>33</v>
@@ -1833,25 +1845,25 @@
     </row>
     <row r="20" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C20" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G20" s="8" t="s">
         <v>126</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>119</v>
       </c>
       <c r="H20" s="8" t="s">
         <v>33</v>
@@ -1859,16 +1871,16 @@
     </row>
     <row r="21" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>52</v>
+        <v>131</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>52</v>
@@ -1877,7 +1889,7 @@
         <v>52</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>33</v>
@@ -1885,25 +1897,25 @@
     </row>
     <row r="22" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>132</v>
+        <v>31</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>133</v>
       </c>
       <c r="D22" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G22" s="8" t="s">
         <v>134</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="G22" s="8" t="s">
-        <v>137</v>
       </c>
       <c r="H22" s="8" t="s">
         <v>33</v>
@@ -1911,25 +1923,25 @@
     </row>
     <row r="23" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C23" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E23" s="3" t="s">
+      <c r="F23" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="G23" s="3" t="s">
         <v>141</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>142</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>33</v>
@@ -1937,19 +1949,19 @@
     </row>
     <row r="24" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="B24" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="C24" s="8" t="s">
+      <c r="D24" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E24" s="8" t="s">
         <v>144</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>135</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>145</v>
@@ -1966,22 +1978,22 @@
         <v>147</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="D25" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="F25" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E25" s="3" t="s">
+      <c r="G25" s="3" t="s">
         <v>150</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>152</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>33</v>
@@ -1989,19 +2001,19 @@
     </row>
     <row r="26" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="C26" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="B26" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="C26" s="8" t="s">
+      <c r="D26" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E26" s="8" t="s">
         <v>154</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>52</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>155</v>
@@ -2018,7 +2030,7 @@
         <v>157</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>158</v>
@@ -2027,13 +2039,13 @@
         <v>52</v>
       </c>
       <c r="E27" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F27" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="G27" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="G27" s="3" t="s">
-        <v>156</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>33</v>
@@ -2044,7 +2056,7 @@
         <v>161</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>162</v>
@@ -2053,13 +2065,13 @@
         <v>52</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>52</v>
+        <v>163</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="H28" s="8" t="s">
         <v>33</v>
@@ -2067,13 +2079,13 @@
     </row>
     <row r="29" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>52</v>
@@ -2082,7 +2094,7 @@
         <v>52</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G29" s="3" t="s">
         <v>156</v>
@@ -2093,25 +2105,25 @@
     </row>
     <row r="30" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>169</v>
+        <v>52</v>
       </c>
       <c r="E30" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F30" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="F30" s="8" t="s">
-        <v>171</v>
-      </c>
       <c r="G30" s="8" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="H30" s="8" t="s">
         <v>33</v>
@@ -2119,25 +2131,25 @@
     </row>
     <row r="31" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D31" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="B31" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C31" s="3" t="s">
+      <c r="E31" s="3" t="s">
         <v>174</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>52</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>175</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>152</v>
+        <v>176</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>33</v>
@@ -2145,13 +2157,13 @@
     </row>
     <row r="32" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B32" s="8" t="s">
         <v>27</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D32" s="8" t="s">
         <v>52</v>
@@ -2160,10 +2172,10 @@
         <v>52</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>179</v>
+        <v>156</v>
       </c>
       <c r="H32" s="8" t="s">
         <v>33</v>
@@ -2174,22 +2186,22 @@
         <v>180</v>
       </c>
       <c r="B33" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="D33" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="D33" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F33" s="3" t="s">
+      <c r="G33" s="3" t="s">
         <v>183</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>179</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>33</v>
@@ -2200,10 +2212,10 @@
         <v>184</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D34" s="8" t="s">
         <v>52</v>
@@ -2212,10 +2224,10 @@
         <v>52</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="H34" s="8" t="s">
         <v>33</v>
@@ -2223,13 +2235,13 @@
     </row>
     <row r="35" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>31</v>
+        <v>185</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>52</v>
@@ -2238,10 +2250,10 @@
         <v>52</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>141</v>
+        <v>182</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>33</v>
@@ -2249,13 +2261,13 @@
     </row>
     <row r="36" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B36" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D36" s="8" t="s">
         <v>52</v>
@@ -2264,7 +2276,7 @@
         <v>52</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>191</v>
+        <v>145</v>
       </c>
       <c r="G36" s="8" t="s">
         <v>192</v>
@@ -2290,10 +2302,10 @@
         <v>52</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>33</v>
@@ -2301,25 +2313,25 @@
     </row>
     <row r="38" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F38" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="B38" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C38" s="8" t="s">
+      <c r="G38" s="8" t="s">
         <v>196</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="F38" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="G38" s="8" t="s">
-        <v>192</v>
       </c>
       <c r="H38" s="8" t="s">
         <v>33</v>
@@ -2327,13 +2339,13 @@
     </row>
     <row r="39" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>132</v>
+        <v>27</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>52</v>
@@ -2342,10 +2354,10 @@
         <v>52</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="H39" s="3" t="s">
         <v>33</v>
@@ -2353,25 +2365,25 @@
     </row>
     <row r="40" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>27</v>
+        <v>136</v>
       </c>
       <c r="C40" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F40" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="D40" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="F40" s="8" t="s">
-        <v>191</v>
-      </c>
       <c r="G40" s="8" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="H40" s="8" t="s">
         <v>33</v>
@@ -2379,13 +2391,13 @@
     </row>
     <row r="41" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>27</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>52</v>
@@ -2394,12 +2406,38 @@
         <v>52</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="H41" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="G42" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="H42" s="8" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2421,15 +2459,15 @@
   <sheetData>
     <row r="1" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="B2" s="5">
         <f>COUNTA('Code Register'!A2:A400)</f>
@@ -2437,7 +2475,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B3" s="5">
         <f>COUNTIF('Code Register'!B2:B400,"Service")</f>
@@ -2445,7 +2483,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B4" s="5">
         <f>COUNTIF('Code Register'!B2:B400,"Renderer")</f>
@@ -2453,7 +2491,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B5" s="5">
         <f>COUNTIF('Code Register'!B2:B400,"Tooling")</f>
@@ -2461,7 +2499,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B6" s="5">
         <f>COUNTIF('Code Register'!H2:H400,"Done")</f>
@@ -2469,7 +2507,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B7" s="5">
         <f>ROUND(COUNTIF('Code Register'!H2:H400,"Done")/COUNTA('Code Register'!A2:A400)*100,1)</f>

</xml_diff>